<commit_message>
Parental leave updates 1
</commit_message>
<xml_diff>
--- a/data/echoMRI/Kotz10072025.xlsx
+++ b/data/echoMRI/Kotz10072025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
   <workbookPr backupFile="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carosandovalcaballero/Documents/GitHub/data/data/echoMRI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carosandovalcab/Documents/GitHub/data/data/echoMRI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB38DD3-D3DD-B44B-84F8-5ABC3571D494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AED0FFAE-3EAA-8A48-B807-570831655560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4300" yWindow="2120" windowWidth="29400" windowHeight="16160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtractedScans" sheetId="1" r:id="rId1"/>
@@ -860,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>315</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1498,7 +1498,7 @@
         <v>1</v>
       </c>
       <c r="I30">
-        <v>317</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="31" spans="1:9">

</xml_diff>